<commit_message>
edit device config files
</commit_message>
<xml_diff>
--- a/01_server_setup/03.ip_address_management/IPAM.xlsx
+++ b/01_server_setup/03.ip_address_management/IPAM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Git_Projects\Network-Automation-Lab\01.server_setup\03.ip_address_management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://georgebrowncollege-my.sharepoint.com/personal/101572831_georgebrown_ca/Documents/Document/IT Files/GitHub Projects/Network-Automation-Lab/01_server_setup/03.ip_address_management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD29EAD9-D19A-4A3C-A08A-5C7C77B20DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{FD29EAD9-D19A-4A3C-A08A-5C7C77B20DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{726CAAF4-EE61-4CDA-B53A-17D31759580E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8C872FB1-40B1-4F13-9BAC-9C3F2D991F53}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="140">
   <si>
     <t>S/N</t>
   </si>
@@ -71,9 +71,6 @@
     <t>CSW2</t>
   </si>
   <si>
-    <t>e1/1</t>
-  </si>
-  <si>
     <t>DSW1</t>
   </si>
   <si>
@@ -447,6 +444,18 @@
   </si>
   <si>
     <t>192.168.2.237/24</t>
+  </si>
+  <si>
+    <t>10.0.110.2</t>
+  </si>
+  <si>
+    <t>e0/3 (EthChannel to CSW2)</t>
+  </si>
+  <si>
+    <t>to DSW2 (Etherchannel)</t>
+  </si>
+  <si>
+    <t>to DSW1 (Etherchannel)</t>
   </si>
 </sst>
 </file>
@@ -470,12 +479,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="15">
@@ -684,7 +699,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -734,6 +749,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -760,6 +781,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1095,7 +1134,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50FBE97E-7632-47FC-9D06-F6D10431D555}">
-  <dimension ref="B1:F55"/>
+  <dimension ref="B1:F56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
@@ -1110,808 +1149,819 @@
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="20">
+      <c r="B3" s="22">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="21"/>
-      <c r="C4" s="18"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="20"/>
       <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="8" t="s">
+    </row>
+    <row r="5" spans="2:6" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="24"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="2:6" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="22"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="16" t="s">
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="22">
+        <v>2</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="23"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="24"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="20">
-        <v>2</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="21"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="22"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="3" t="s">
+      <c r="F8" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F8" s="8" t="s">
+    </row>
+    <row r="9" spans="2:6" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="22">
+        <v>3</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="9" spans="2:6" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="20">
-        <v>3</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>37</v>
-      </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="21"/>
-      <c r="C10" s="18"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="20"/>
       <c r="D10" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="8" t="s">
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="23"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="29" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="21"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="8" t="s">
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="29" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="21"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="3" t="s">
+      <c r="F12" s="30" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="24"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="25">
+        <v>4</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="26"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="22"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="23">
-        <v>4</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F14" s="8" t="s">
+      <c r="E15" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="24"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>48</v>
-      </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="24"/>
-      <c r="C16" s="18"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="20"/>
       <c r="D16" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="8" t="s">
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="26"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="24"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="26"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="24"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="8" t="s">
+    </row>
+    <row r="19" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B19" s="27"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="19" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19" s="25"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="16" t="s">
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="22">
+        <v>5</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="23"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="23"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="30" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B23" s="23"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="24"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F19" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="20">
-        <v>5</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="21"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="21"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B23" s="21"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F23" s="8" t="s">
+      <c r="F24" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="22"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="F24" s="8" t="s">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="22">
+        <v>6</v>
+      </c>
+      <c r="C25" s="19" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="20">
-        <v>6</v>
-      </c>
-      <c r="C25" s="17" t="s">
+      <c r="D25" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="F25" s="8" t="s">
-        <v>71</v>
-      </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="21"/>
-      <c r="C26" s="18"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="20"/>
       <c r="D26" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F26" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="F26" s="8" t="s">
-        <v>73</v>
-      </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="21"/>
-      <c r="C27" s="18"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="20"/>
       <c r="D27" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F27" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="F27" s="8" t="s">
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="24"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B29" s="18"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="22">
+        <v>7</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="22"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E28" s="1" t="s">
+      <c r="E30" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="23"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="F31" s="33" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B32" s="23"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="23"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="24"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F28" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="20">
-        <v>7</v>
-      </c>
-      <c r="C29" s="17" t="s">
+      <c r="F34" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="22">
+        <v>8</v>
+      </c>
+      <c r="C35" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="21"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="21"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="3" t="s">
+      <c r="D35" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B36" s="23"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="21"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="3" t="s">
+      <c r="E36" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B37" s="24"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="22">
         <v>9</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="22"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="20">
-        <v>8</v>
-      </c>
-      <c r="C34" s="17" t="s">
+      <c r="C38" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="21"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="3" t="s">
+      <c r="D38" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="23"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="24"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B41" s="22">
+        <v>10</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B42" s="23"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B43" s="24"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B44" s="22">
+        <v>11</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B45" s="23">
+        <v>11</v>
+      </c>
+      <c r="C45" s="20"/>
+      <c r="D45" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B46" s="24">
+        <v>11</v>
+      </c>
+      <c r="C46" s="21"/>
+      <c r="D46" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B47" s="22">
+        <v>12</v>
+      </c>
+      <c r="C47" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B48" s="23">
+        <v>12</v>
+      </c>
+      <c r="C48" s="20"/>
+      <c r="D48" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B49" s="24">
+        <v>12</v>
+      </c>
+      <c r="C49" s="21"/>
+      <c r="D49" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B50" s="22">
+        <v>13</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B51" s="23"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B52" s="24"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B53" s="22">
+        <v>14</v>
+      </c>
+      <c r="C53" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F53" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B54" s="23">
+        <v>14</v>
+      </c>
+      <c r="C54" s="20"/>
+      <c r="D54" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="F35" s="8" t="s">
+      <c r="E54" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B55" s="24">
+        <v>14</v>
+      </c>
+      <c r="C55" s="21"/>
+      <c r="D55" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B36" s="22"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="20">
-        <v>9</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F37" s="8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="21"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E38" s="1" t="s">
+      <c r="E55" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F55" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="F38" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" s="22"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="20">
-        <v>10</v>
-      </c>
-      <c r="C40" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F40" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="21"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="22"/>
-      <c r="C42" s="19"/>
-      <c r="D42" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="F42" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="20">
-        <v>11</v>
-      </c>
-      <c r="C43" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="F43" s="8" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B44" s="21">
-        <v>11</v>
-      </c>
-      <c r="C44" s="18"/>
-      <c r="D44" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="F44" s="8" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B45" s="22">
-        <v>11</v>
-      </c>
-      <c r="C45" s="19"/>
-      <c r="D45" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B46" s="20">
-        <v>12</v>
-      </c>
-      <c r="C46" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="F46" s="8" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B47" s="21">
-        <v>12</v>
-      </c>
-      <c r="C47" s="18"/>
-      <c r="D47" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F47" s="8" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B48" s="22">
-        <v>12</v>
-      </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="F48" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B49" s="20">
-        <v>13</v>
-      </c>
-      <c r="C49" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="F49" s="8" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B50" s="21"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F50" s="8" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B51" s="22"/>
-      <c r="C51" s="19"/>
-      <c r="D51" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F51" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B52" s="20">
-        <v>14</v>
-      </c>
-      <c r="C52" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="F52" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B53" s="21">
-        <v>14</v>
-      </c>
-      <c r="C53" s="18"/>
-      <c r="D53" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E53" s="1" t="s">
+    </row>
+    <row r="56" spans="2:6" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="F53" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B54" s="22">
-        <v>14</v>
-      </c>
-      <c r="C54" s="19"/>
-      <c r="D54" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F54" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="9" t="s">
+      <c r="C56" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="D56" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="D55" s="10" t="s">
+      <c r="E56" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="E55" s="11" t="s">
+      <c r="F56" s="12" t="s">
         <v>120</v>
-      </c>
-      <c r="F55" s="12" t="s">
-        <v>121</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="C53:C55"/>
+    <mergeCell ref="B53:B55"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C30:C34"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C14:C19"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="C20:C24"/>
+    <mergeCell ref="B20:B24"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="B25:B28"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C9:C13"/>
     <mergeCell ref="B9:B13"/>
-    <mergeCell ref="C14:C19"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="C20:C24"/>
-    <mergeCell ref="B20:B24"/>
-    <mergeCell ref="C25:C28"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="C29:C33"/>
-    <mergeCell ref="B29:B33"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B37:B39"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="B49:B51"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="B52:B54"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="B46:B48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>